<commit_message>
kørselsaftale, styresystem tilføjet excelark
</commit_message>
<xml_diff>
--- a/P6data/VL.xlsx
+++ b/P6data/VL.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ebk\Trafikstyring V2\P6data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8875962C-DEC0-4266-814D-172AD9BBA12A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E891819-5B29-41AE-AE0F-BABB25DD066C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="570" windowWidth="29040" windowHeight="16830" xr2:uid="{E7DE5B6D-17B1-4BBB-8342-C7DA09B36074}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="27">
   <si>
     <t>24-2267</t>
   </si>
@@ -111,6 +111,12 @@
   </si>
   <si>
     <t>CROSSER</t>
+  </si>
+  <si>
+    <t>Kørselsaftale</t>
+  </si>
+  <si>
+    <t>Styresystem</t>
   </si>
 </sst>
 </file>
@@ -504,20 +510,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2422EC17-15C8-4726-B31A-3667559F39F4}">
-  <dimension ref="A1:T7"/>
+  <dimension ref="A1:V7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="22.7109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="22.7109375" customWidth="1"/>
+    <col min="3" max="4" width="16.85546875" customWidth="1"/>
+    <col min="6" max="6" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="14.28515625" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="22.7109375" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="22.7109375" customWidth="1"/>
     <col min="15" max="15" width="22.7109375" bestFit="1" customWidth="1"/>
@@ -526,9 +531,11 @@
     <col min="18" max="18" width="22.7109375" customWidth="1"/>
     <col min="19" max="19" width="22.7109375" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="22.7109375" customWidth="1"/>
+    <col min="21" max="21" width="22.7109375" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="22.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>1</v>
       </c>
@@ -536,34 +543,34 @@
         <v>2</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="K1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>10</v>
-      </c>
-      <c r="K1" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="L1" s="2" t="s">
-        <v>11</v>
       </c>
       <c r="M1" s="2" t="s">
         <v>11</v>
@@ -589,376 +596,418 @@
       <c r="T1" s="2" t="s">
         <v>11</v>
       </c>
+      <c r="U1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="V1" s="2" t="s">
+        <v>11</v>
+      </c>
     </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="2">
         <v>31400</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>12</v>
+      <c r="C2" s="2">
+        <v>3400</v>
+      </c>
+      <c r="D2" s="2">
+        <v>1</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F2" s="2">
+      <c r="F2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H2" s="2">
         <v>70112210</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="I2" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="H2" s="2">
-        <v>31400</v>
-      </c>
-      <c r="I2" s="2">
-        <v>31400</v>
-      </c>
-      <c r="J2" s="2" t="s">
+      <c r="J2" s="2">
+        <v>31400</v>
+      </c>
+      <c r="K2" s="2">
+        <v>31400</v>
+      </c>
+      <c r="L2" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="K2" s="2" t="s">
+      <c r="M2" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="L2" s="2" t="s">
+      <c r="N2" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="M2" s="2" t="s">
+      <c r="O2" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="N2" s="2" t="s">
+      <c r="P2" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="O2" s="2" t="s">
+      <c r="Q2" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="P2" s="2" t="s">
+      <c r="R2" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="Q2" s="2" t="s">
+      <c r="S2" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="R2" s="2" t="s">
+      <c r="T2" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="S2" s="2" t="s">
+      <c r="U2" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="T2" s="2" t="s">
+      <c r="V2" s="2" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B3" s="2">
         <v>31400</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>12</v>
+      <c r="C3" s="2">
+        <v>3400</v>
+      </c>
+      <c r="D3" s="2">
+        <v>1</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F3" s="2">
+      <c r="F3" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H3" s="2">
         <v>70112210</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="I3" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="H3" s="2">
-        <v>31400</v>
-      </c>
-      <c r="I3" s="2">
-        <v>31400</v>
-      </c>
-      <c r="J3" s="2" t="s">
+      <c r="J3" s="2">
+        <v>31400</v>
+      </c>
+      <c r="K3" s="2">
+        <v>31400</v>
+      </c>
+      <c r="L3" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="K3" s="2" t="s">
+      <c r="M3" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="L3" s="2" t="s">
+      <c r="N3" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="M3" s="2" t="s">
+      <c r="O3" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="N3" s="2" t="s">
+      <c r="P3" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="O3" s="2" t="s">
+      <c r="Q3" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="P3" s="2" t="s">
+      <c r="R3" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="Q3" s="2" t="s">
+      <c r="S3" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="R3" s="2" t="s">
+      <c r="T3" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="S3" s="2" t="s">
+      <c r="U3" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="T3" s="2" t="s">
+      <c r="V3" s="2" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B4" s="2">
         <v>31400</v>
       </c>
-      <c r="C4" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>12</v>
+      <c r="C4" s="2">
+        <v>3400</v>
+      </c>
+      <c r="D4" s="2">
+        <v>1</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F4" s="2">
+      <c r="F4" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H4" s="2">
         <v>70112210</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="I4" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="H4" s="2">
-        <v>31400</v>
-      </c>
-      <c r="I4" s="2">
-        <v>31400</v>
-      </c>
-      <c r="J4" s="2" t="s">
+      <c r="J4" s="2">
+        <v>31400</v>
+      </c>
+      <c r="K4" s="2">
+        <v>31400</v>
+      </c>
+      <c r="L4" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="K4" s="2" t="s">
+      <c r="M4" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="L4" s="2" t="s">
+      <c r="N4" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="M4" s="2" t="s">
+      <c r="O4" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="N4" s="2" t="s">
+      <c r="P4" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="O4" s="2" t="s">
+      <c r="Q4" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="P4" s="2" t="s">
+      <c r="R4" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="Q4" s="2" t="s">
+      <c r="S4" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="R4" s="2" t="s">
+      <c r="T4" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="S4" s="2" t="s">
+      <c r="U4" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="T4" s="2" t="s">
+      <c r="V4" s="2" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B5" s="2">
         <v>31400</v>
       </c>
-      <c r="C5" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>12</v>
+      <c r="C5" s="2">
+        <v>3400</v>
+      </c>
+      <c r="D5" s="2">
+        <v>1</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F5" s="2">
+      <c r="F5" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H5" s="2">
         <v>70112210</v>
       </c>
-      <c r="G5" s="2" t="s">
+      <c r="I5" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="H5" s="2">
-        <v>31400</v>
-      </c>
-      <c r="I5" s="2">
-        <v>31400</v>
-      </c>
-      <c r="J5" s="2" t="s">
+      <c r="J5" s="2">
+        <v>31400</v>
+      </c>
+      <c r="K5" s="2">
+        <v>31400</v>
+      </c>
+      <c r="L5" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="K5" s="2" t="s">
+      <c r="M5" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="L5" s="2" t="s">
+      <c r="N5" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="M5" s="2" t="s">
+      <c r="O5" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="N5" s="2" t="s">
+      <c r="P5" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="O5" s="2" t="s">
+      <c r="Q5" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="P5" s="2" t="s">
+      <c r="R5" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="Q5" s="2" t="s">
+      <c r="S5" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="R5" s="2" t="s">
+      <c r="T5" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="S5" s="2" t="s">
+      <c r="U5" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="T5" s="2" t="s">
+      <c r="V5" s="2" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B6" s="2">
         <v>31400</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>12</v>
+      <c r="C6" s="2">
+        <v>3400</v>
+      </c>
+      <c r="D6" s="2">
+        <v>1</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F6" s="2">
+      <c r="F6" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H6" s="2">
         <v>70112210</v>
       </c>
-      <c r="G6" s="2" t="s">
+      <c r="I6" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="H6" s="2">
-        <v>31400</v>
-      </c>
-      <c r="I6" s="2">
-        <v>31400</v>
-      </c>
-      <c r="J6" s="2" t="s">
+      <c r="J6" s="2">
+        <v>31400</v>
+      </c>
+      <c r="K6" s="2">
+        <v>31400</v>
+      </c>
+      <c r="L6" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="K6" s="2" t="s">
+      <c r="M6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="L6" s="2" t="s">
+      <c r="N6" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="M6" s="2" t="s">
+      <c r="O6" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="N6" s="2" t="s">
+      <c r="P6" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="O6" s="2" t="s">
+      <c r="Q6" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="P6" s="2" t="s">
+      <c r="R6" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="Q6" s="2" t="s">
+      <c r="S6" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="R6" s="2" t="s">
+      <c r="T6" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="S6" s="2" t="s">
+      <c r="U6" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="T6" s="2" t="s">
+      <c r="V6" s="2" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B7" s="2">
         <v>31400</v>
       </c>
-      <c r="C7" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>12</v>
+      <c r="C7" s="2">
+        <v>3400</v>
+      </c>
+      <c r="D7" s="2">
+        <v>1</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F7" s="2">
+      <c r="F7" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H7" s="2">
         <v>70112210</v>
       </c>
-      <c r="G7" s="2" t="s">
+      <c r="I7" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="H7" s="2">
-        <v>31400</v>
-      </c>
-      <c r="I7" s="2">
-        <v>31400</v>
-      </c>
-      <c r="J7" s="2" t="s">
+      <c r="J7" s="2">
+        <v>31400</v>
+      </c>
+      <c r="K7" s="2">
+        <v>31400</v>
+      </c>
+      <c r="L7" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="K7" s="2" t="s">
+      <c r="M7" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="L7" s="2" t="s">
+      <c r="N7" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="M7" s="2" t="s">
+      <c r="O7" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="N7" s="2" t="s">
+      <c r="P7" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="O7" s="2" t="s">
+      <c r="Q7" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="P7" s="2" t="s">
+      <c r="R7" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="Q7" s="2" t="s">
+      <c r="S7" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="R7" s="2" t="s">
+      <c r="T7" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="S7" s="2" t="s">
+      <c r="U7" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="T7" s="2" t="s">
+      <c r="V7" s="2" t="s">
         <v>24</v>
       </c>
     </row>

</xml_diff>

<commit_message>
indlæs data på vognløbsObj
</commit_message>
<xml_diff>
--- a/P6data/VL.xlsx
+++ b/P6data/VL.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ebk\Trafikstyring V2\P6data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E891819-5B29-41AE-AE0F-BABB25DD066C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E74E3243-9153-443E-B0AA-276E964CAFC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="570" windowWidth="29040" windowHeight="16830" xr2:uid="{E7DE5B6D-17B1-4BBB-8342-C7DA09B36074}"/>
   </bookViews>
   <sheets>
     <sheet name="Ark1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" refMode="R1C1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="28">
   <si>
     <t>24-2267</t>
   </si>
@@ -56,9 +56,6 @@
     <t>Hjemzone</t>
   </si>
   <si>
-    <t>Mobilnr</t>
-  </si>
-  <si>
     <t>Vognløbskategori</t>
   </si>
   <si>
@@ -117,6 +114,12 @@
   </si>
   <si>
     <t>Styresystem</t>
+  </si>
+  <si>
+    <t>MobilnrChf</t>
+  </si>
+  <si>
+    <t>asd</t>
   </si>
 </sst>
 </file>
@@ -543,10 +546,10 @@
         <v>2</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>25</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>26</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>3</v>
@@ -558,49 +561,49 @@
         <v>5</v>
       </c>
       <c r="H1" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="I1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="K1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="M1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="M1" s="2" t="s">
-        <v>11</v>
-      </c>
       <c r="N1" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="O1" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="P1" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="Q1" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="R1" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="S1" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="T1" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="U1" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="V1" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:22" x14ac:dyDescent="0.25">
@@ -617,19 +620,19 @@
         <v>1</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H2" s="2">
         <v>70112210</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="J2" s="2">
         <v>31400</v>
@@ -638,37 +641,37 @@
         <v>31400</v>
       </c>
       <c r="L2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="M2" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="M2" s="2" t="s">
+      <c r="N2" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="N2" s="2" t="s">
+      <c r="O2" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="O2" s="2" t="s">
+      <c r="P2" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="P2" s="2" t="s">
+      <c r="Q2" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="Q2" s="2" t="s">
+      <c r="R2" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="R2" s="2" t="s">
+      <c r="S2" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="S2" s="2" t="s">
+      <c r="T2" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="T2" s="2" t="s">
+      <c r="U2" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="U2" s="2" t="s">
+      <c r="V2" s="2" t="s">
         <v>23</v>
-      </c>
-      <c r="V2" s="2" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="3" spans="1:22" x14ac:dyDescent="0.25">
@@ -676,67 +679,67 @@
         <v>0</v>
       </c>
       <c r="B3" s="2">
-        <v>31400</v>
+        <v>31401</v>
       </c>
       <c r="C3" s="2">
         <v>3400</v>
       </c>
       <c r="D3" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H3" s="2">
         <v>70112210</v>
       </c>
-      <c r="I3" s="2" t="s">
+      <c r="I3" s="2">
+        <v>2</v>
+      </c>
+      <c r="J3" s="2">
+        <v>23</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="L3" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="J3" s="2">
-        <v>31400</v>
-      </c>
-      <c r="K3" s="2">
-        <v>31400</v>
-      </c>
-      <c r="L3" s="2" t="s">
+      <c r="M3" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="M3" s="2" t="s">
+      <c r="N3" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="N3" s="2" t="s">
+      <c r="O3" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="O3" s="2" t="s">
+      <c r="P3" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="P3" s="2" t="s">
+      <c r="Q3" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="Q3" s="2" t="s">
+      <c r="R3" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="R3" s="2" t="s">
+      <c r="S3" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="S3" s="2" t="s">
+      <c r="T3" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="T3" s="2" t="s">
+      <c r="U3" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="U3" s="2" t="s">
+      <c r="V3" s="2" t="s">
         <v>23</v>
-      </c>
-      <c r="V3" s="2" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:22" x14ac:dyDescent="0.25">
@@ -744,67 +747,67 @@
         <v>0</v>
       </c>
       <c r="B4" s="2">
-        <v>31400</v>
+        <v>31402</v>
       </c>
       <c r="C4" s="2">
         <v>3400</v>
       </c>
       <c r="D4" s="2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H4" s="2">
         <v>70112210</v>
       </c>
-      <c r="I4" s="2" t="s">
+      <c r="I4" s="2">
+        <v>3</v>
+      </c>
+      <c r="J4" s="2">
+        <v>34324</v>
+      </c>
+      <c r="K4" s="2">
+        <v>3</v>
+      </c>
+      <c r="L4" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="J4" s="2">
-        <v>31400</v>
-      </c>
-      <c r="K4" s="2">
-        <v>31400</v>
-      </c>
-      <c r="L4" s="2" t="s">
+      <c r="M4" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="M4" s="2" t="s">
+      <c r="N4" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="N4" s="2" t="s">
+      <c r="O4" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="O4" s="2" t="s">
+      <c r="P4" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="P4" s="2" t="s">
+      <c r="Q4" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="Q4" s="2" t="s">
+      <c r="R4" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="R4" s="2" t="s">
+      <c r="S4" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="S4" s="2" t="s">
+      <c r="T4" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="T4" s="2" t="s">
+      <c r="U4" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="U4" s="2" t="s">
+      <c r="V4" s="2" t="s">
         <v>23</v>
-      </c>
-      <c r="V4" s="2" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="5" spans="1:22" x14ac:dyDescent="0.25">
@@ -812,67 +815,67 @@
         <v>0</v>
       </c>
       <c r="B5" s="2">
-        <v>31400</v>
+        <v>31403</v>
       </c>
       <c r="C5" s="2">
         <v>3400</v>
       </c>
       <c r="D5" s="2">
-        <v>1</v>
+        <v>54</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H5" s="2">
         <v>70112210</v>
       </c>
-      <c r="I5" s="2" t="s">
+      <c r="I5" s="2">
+        <v>4</v>
+      </c>
+      <c r="J5" s="2">
+        <v>3324</v>
+      </c>
+      <c r="K5" s="2">
+        <v>21</v>
+      </c>
+      <c r="L5" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="J5" s="2">
-        <v>31400</v>
-      </c>
-      <c r="K5" s="2">
-        <v>31400</v>
-      </c>
-      <c r="L5" s="2" t="s">
+      <c r="M5" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="M5" s="2" t="s">
+      <c r="N5" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="N5" s="2" t="s">
+      <c r="O5" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="O5" s="2" t="s">
+      <c r="P5" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="P5" s="2" t="s">
+      <c r="Q5" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="Q5" s="2" t="s">
+      <c r="R5" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="R5" s="2" t="s">
+      <c r="S5" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="S5" s="2" t="s">
+      <c r="T5" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="T5" s="2" t="s">
+      <c r="U5" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="U5" s="2" t="s">
+      <c r="V5" s="2" t="s">
         <v>23</v>
-      </c>
-      <c r="V5" s="2" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="6" spans="1:22" x14ac:dyDescent="0.25">
@@ -880,67 +883,67 @@
         <v>0</v>
       </c>
       <c r="B6" s="2">
-        <v>31400</v>
+        <v>31404</v>
       </c>
       <c r="C6" s="2">
         <v>3400</v>
       </c>
       <c r="D6" s="2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H6" s="2">
         <v>70112210</v>
       </c>
-      <c r="I6" s="2" t="s">
+      <c r="I6" s="2">
+        <v>5</v>
+      </c>
+      <c r="J6" s="2">
+        <v>121</v>
+      </c>
+      <c r="K6" s="2">
+        <v>43</v>
+      </c>
+      <c r="L6" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="J6" s="2">
-        <v>31400</v>
-      </c>
-      <c r="K6" s="2">
-        <v>31400</v>
-      </c>
-      <c r="L6" s="2" t="s">
+      <c r="M6" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="M6" s="2" t="s">
+      <c r="N6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="N6" s="2" t="s">
+      <c r="O6" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="O6" s="2" t="s">
+      <c r="P6" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="P6" s="2" t="s">
+      <c r="Q6" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="Q6" s="2" t="s">
+      <c r="R6" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="R6" s="2" t="s">
+      <c r="S6" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="S6" s="2" t="s">
+      <c r="T6" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="T6" s="2" t="s">
+      <c r="U6" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="U6" s="2" t="s">
+      <c r="V6" s="2" t="s">
         <v>23</v>
-      </c>
-      <c r="V6" s="2" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="7" spans="1:22" x14ac:dyDescent="0.25">
@@ -948,67 +951,67 @@
         <v>0</v>
       </c>
       <c r="B7" s="2">
-        <v>31400</v>
+        <v>31405</v>
       </c>
       <c r="C7" s="2">
         <v>3400</v>
       </c>
       <c r="D7" s="2">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H7" s="2">
         <v>70112210</v>
       </c>
-      <c r="I7" s="2" t="s">
+      <c r="I7" s="2">
+        <v>53</v>
+      </c>
+      <c r="J7" s="2">
+        <v>23</v>
+      </c>
+      <c r="K7" s="2">
+        <v>5</v>
+      </c>
+      <c r="L7" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="J7" s="2">
-        <v>31400</v>
-      </c>
-      <c r="K7" s="2">
-        <v>31400</v>
-      </c>
-      <c r="L7" s="2" t="s">
+      <c r="M7" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="M7" s="2" t="s">
+      <c r="N7" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="N7" s="2" t="s">
+      <c r="O7" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="O7" s="2" t="s">
+      <c r="P7" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="P7" s="2" t="s">
+      <c r="Q7" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="Q7" s="2" t="s">
+      <c r="R7" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="R7" s="2" t="s">
+      <c r="S7" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="S7" s="2" t="s">
+      <c r="T7" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="T7" s="2" t="s">
+      <c r="U7" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="U7" s="2" t="s">
+      <c r="V7" s="2" t="s">
         <v>23</v>
-      </c>
-      <c r="V7" s="2" t="s">
-        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fiks listview, indsæt korrekt rækkefølge, fra bunden
</commit_message>
<xml_diff>
--- a/P6data/VL.xlsx
+++ b/P6data/VL.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ebk\Trafikstyring V2\P6data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E74E3243-9153-443E-B0AA-276E964CAFC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0678D47B-6860-4BB5-BBDA-55DC619D9763}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="570" windowWidth="29040" windowHeight="16830" xr2:uid="{E7DE5B6D-17B1-4BBB-8342-C7DA09B36074}"/>
   </bookViews>
@@ -611,7 +611,7 @@
         <v>0</v>
       </c>
       <c r="B2" s="2">
-        <v>31400</v>
+        <v>12</v>
       </c>
       <c r="C2" s="2">
         <v>3400</v>

</xml_diff>